<commit_message>
update#4-update removed job filter excels from email
</commit_message>
<xml_diff>
--- a/job-filters.xlsx
+++ b/job-filters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Shubham\fiverr\raikaphotograph\task-schedular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E1579B3-00CA-4EED-A5A8-A782D59BE46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC15EBB1-5B75-4B17-B91A-3A466E8CD984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -288,7 +288,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -650,7 +650,7 @@
         <v>26</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>17</v>

</xml_diff>